<commit_message>
vault backup: 2026-09-28 16:14:49
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
+++ b/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Методологии и проектирование ИС\ДЗ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB261146-2A3F-4018-9DDA-115243CF676A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B941381F-B6C3-4659-8EEB-AAB8795FFF3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
   <si>
     <t>Наименование</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>Сотрудник</t>
+  </si>
+  <si>
+    <t>Инструменты</t>
   </si>
 </sst>
 </file>
@@ -131,7 +134,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -140,6 +143,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -162,6 +180,21 @@
         <color indexed="64"/>
       </right>
       <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -325,6 +358,45 @@
       </right>
       <top/>
       <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -333,12 +405,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
@@ -347,58 +416,67 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -799,7 +877,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="14"/>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="20" t="s">
         <v>15</v>
       </c>
     </row>
@@ -808,7 +886,7 @@
         <v>13</v>
       </c>
       <c r="B10" s="16"/>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="18" t="s">
         <v>15</v>
       </c>
     </row>
@@ -817,7 +895,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="16"/>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="18" t="s">
         <v>15</v>
       </c>
     </row>
@@ -826,7 +904,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="16"/>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="18" t="s">
         <v>17</v>
       </c>
     </row>
@@ -835,7 +913,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="16"/>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="18" t="s">
         <v>17</v>
       </c>
     </row>
@@ -844,7 +922,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="16"/>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="18" t="s">
         <v>17</v>
       </c>
     </row>
@@ -853,26 +931,34 @@
         <v>16</v>
       </c>
       <c r="B15" s="16"/>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="18" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="15"/>
+      <c r="A16" s="15" t="s">
+        <v>20</v>
+      </c>
       <c r="B16" s="16"/>
-      <c r="C16" s="17"/>
+      <c r="C16" s="17" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="15"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="17"/>
+      <c r="A17" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="18" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="20" t="s">
+      <c r="B18" s="22"/>
+      <c r="C18" s="23" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-28 16:19:40
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
+++ b/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Методологии и проектирование ИС\ДЗ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B941381F-B6C3-4659-8EEB-AAB8795FFF3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF83B64-7321-4C22-86FD-41948D23E516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
   <si>
     <t>Наименование</t>
   </si>
@@ -102,6 +102,12 @@
   </si>
   <si>
     <t>Инструменты</t>
+  </si>
+  <si>
+    <t>Выход</t>
+  </si>
+  <si>
+    <t>Прибыль</t>
   </si>
 </sst>
 </file>
@@ -134,7 +140,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -401,11 +407,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -477,6 +496,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -813,7 +835,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B15018C-9950-4198-9E61-792B87EB61C3}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.109375" customWidth="1"/>
@@ -953,13 +975,31 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="23" t="s">
-        <v>18</v>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="19"/>
+      <c r="C18" s="18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="25"/>
+      <c r="C19" s="20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="22"/>
+      <c r="C20" s="23" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-09-28 16:20:54
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
+++ b/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Методологии и проектирование ИС\ДЗ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF83B64-7321-4C22-86FD-41948D23E516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91CABC28-E1C1-45DB-A8CF-9516F51D2462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="A3" sheetId="1" r:id="rId1"/>
+    <sheet name="A31" sheetId="2" r:id="rId2"/>
+    <sheet name="A311" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1009,4 +1011,22 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BC85141-7E3B-47EF-AC56-0B57B5CB3222}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72000FC0-1D0E-4531-A073-6777A317129E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-09-28 16:25:16
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
+++ b/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Методологии и проектирование ИС\ДЗ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91CABC28-E1C1-45DB-A8CF-9516F51D2462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D353A7F1-9445-4DAF-9D3A-D35E3A4E85F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
   </bookViews>
   <sheets>
     <sheet name="A3" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
   <si>
     <t>Наименование</t>
   </si>
@@ -110,6 +110,12 @@
   </si>
   <si>
     <t>Прибыль</t>
+  </si>
+  <si>
+    <t>Выезд</t>
+  </si>
+  <si>
+    <t>Локально</t>
   </si>
 </sst>
 </file>
@@ -1015,9 +1021,42 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BC85141-7E3B-47EF-AC56-0B57B5CB3222}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="2" width="26.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="8"/>
+    </row>
+    <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="4"/>
+    </row>
+    <row r="4" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
vault backup: 2026-09-28 16:32:58
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
+++ b/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Методологии и проектирование ИС\ДЗ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D353A7F1-9445-4DAF-9D3A-D35E3A4E85F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085696E0-AF50-4611-A948-36B4AE68D7C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
   </bookViews>
   <sheets>
-    <sheet name="A3" sheetId="1" r:id="rId1"/>
-    <sheet name="A31" sheetId="2" r:id="rId2"/>
+    <sheet name="A3 &quot;Ремонт&quot;" sheetId="1" r:id="rId1"/>
+    <sheet name="A31 &quot;Диагностирование&quot;" sheetId="2" r:id="rId2"/>
     <sheet name="A311" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="34">
   <si>
     <t>Наименование</t>
   </si>
@@ -55,7 +55,7 @@
     <t>Описание (назначение)</t>
   </si>
   <si>
-    <t>Стрелки диаграммы "Ремонт" (A3)</t>
+    <t>Процессы (работы) диаграммы "Ремонт"</t>
   </si>
   <si>
     <t>Процессы (работы) диаграммы "Ремонт" (A3)</t>
@@ -116,6 +116,33 @@
   </si>
   <si>
     <t>Локально</t>
+  </si>
+  <si>
+    <t>Правила выездной диагностики</t>
+  </si>
+  <si>
+    <t>Правили локальной диагностики</t>
+  </si>
+  <si>
+    <t>Выезд к клиенту</t>
+  </si>
+  <si>
+    <t>Первичное тестирование</t>
+  </si>
+  <si>
+    <t>Ремонт на месте</t>
+  </si>
+  <si>
+    <t>Транспортировка устройства</t>
+  </si>
+  <si>
+    <t>Стрелки диаграммы "Ремонт"</t>
+  </si>
+  <si>
+    <t>Процессы (работы) диаграммы</t>
+  </si>
+  <si>
+    <t>Стрелки диаграммы</t>
   </si>
 </sst>
 </file>
@@ -148,7 +175,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -370,6 +397,19 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -426,14 +466,33 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -491,9 +550,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -503,11 +559,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -852,161 +917,161 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="10"/>
     </row>
     <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="12" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="4"/>
+      <c r="B3" s="6"/>
     </row>
     <row r="4" spans="1:3" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="4"/>
     </row>
     <row r="5" spans="1:3" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6"/>
+      <c r="B5" s="8"/>
     </row>
     <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="8"/>
+      <c r="A7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="10"/>
     </row>
     <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="12" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="20" t="s">
+      <c r="B9" s="16"/>
+      <c r="C9" s="22" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="18" t="s">
+      <c r="B10" s="18"/>
+      <c r="C10" s="20" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="16"/>
-      <c r="C11" s="18" t="s">
+      <c r="B11" s="18"/>
+      <c r="C11" s="20" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="18" t="s">
+      <c r="B12" s="18"/>
+      <c r="C12" s="20" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="18" t="s">
+      <c r="B13" s="18"/>
+      <c r="C13" s="20" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="18" t="s">
+      <c r="B14" s="18"/>
+      <c r="C14" s="20" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="18" t="s">
+      <c r="B15" s="18"/>
+      <c r="C15" s="20" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="17" t="s">
+      <c r="B16" s="18"/>
+      <c r="C16" s="19" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="18" t="s">
+      <c r="B17" s="21"/>
+      <c r="C17" s="20" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="18" t="s">
+      <c r="B18" s="21"/>
+      <c r="C18" s="20" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="20" t="s">
+      <c r="B19" s="27"/>
+      <c r="C19" s="22" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="23" t="s">
+      <c r="B20" s="24"/>
+      <c r="C20" s="25" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1021,41 +1086,143 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BC85141-7E3B-47EF-AC56-0B57B5CB3222}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="8"/>
-    </row>
-    <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="B1" s="10"/>
+    </row>
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="4"/>
-    </row>
-    <row r="4" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
+      <c r="B3" s="6"/>
+    </row>
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="6"/>
+      <c r="B4" s="8"/>
+    </row>
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="10"/>
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="16"/>
+      <c r="C8" s="22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="18"/>
+      <c r="C9" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="C10" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="18"/>
+      <c r="C11" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="18"/>
+      <c r="C13" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="21"/>
+      <c r="C14" s="20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="21"/>
+      <c r="C15" s="20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="24"/>
+      <c r="C16" s="25" t="s">
+        <v>21</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1063,9 +1230,156 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72000FC0-1D0E-4531-A073-6777A317129E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="2" width="26.77734375" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="10"/>
+    </row>
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="29"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="8"/>
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="13"/>
+      <c r="C8" s="10"/>
+    </row>
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="16"/>
+      <c r="C10" s="22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="18"/>
+      <c r="C11" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A13" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="18"/>
+      <c r="C13" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="18"/>
+      <c r="C14" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="18"/>
+      <c r="C15" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="21"/>
+      <c r="C16" s="20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="21"/>
+      <c r="C17" s="20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="24"/>
+      <c r="C18" s="25" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A8:C8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-09-28 16:41:34
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
+++ b/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Методологии и проектирование ИС\ДЗ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085696E0-AF50-4611-A948-36B4AE68D7C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E2826A-7451-4A3E-9215-2BC00EB1618C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="2" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
   </bookViews>
   <sheets>
     <sheet name="A3 &quot;Ремонт&quot;" sheetId="1" r:id="rId1"/>
     <sheet name="A31 &quot;Диагностирование&quot;" sheetId="2" r:id="rId2"/>
-    <sheet name="A311" sheetId="3" r:id="rId3"/>
+    <sheet name="A311 &quot;Выезд&quot;" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="33">
   <si>
     <t>Наименование</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>Процессы (работы) диаграммы "Ремонт"</t>
-  </si>
-  <si>
-    <t>Процессы (работы) диаграммы "Ремонт" (A3)</t>
   </si>
   <si>
     <t>Диагностирование</t>
@@ -918,7 +915,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B1" s="10"/>
     </row>
@@ -932,26 +929,26 @@
     </row>
     <row r="3" spans="1:3" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" s="6"/>
     </row>
     <row r="4" spans="1:3" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" s="4"/>
     </row>
     <row r="5" spans="1:3" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" s="8"/>
     </row>
     <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="10"/>
@@ -969,110 +966,110 @@
     </row>
     <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" s="18"/>
       <c r="C10" s="20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" s="18"/>
       <c r="C15" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" s="18"/>
       <c r="C16" s="19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" s="21"/>
       <c r="C18" s="20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20" s="24"/>
       <c r="C20" s="25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1095,7 +1092,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B1" s="10"/>
     </row>
@@ -1109,20 +1106,20 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="6"/>
     </row>
     <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" s="8"/>
     </row>
     <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="10"/>
@@ -1140,83 +1137,83 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" s="16"/>
       <c r="C8" s="22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="18"/>
       <c r="C9" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="18"/>
       <c r="C10" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="21"/>
       <c r="C15" s="20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="24"/>
       <c r="C16" s="25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1253,32 +1250,32 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B3" s="29"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" s="2"/>
     </row>
     <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B6" s="8"/>
     </row>
     <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="10"/>
@@ -1296,83 +1293,83 @@
     </row>
     <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="16"/>
       <c r="C10" s="22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B15" s="18"/>
       <c r="C15" s="19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18" s="24"/>
       <c r="C18" s="25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-09-28 17:08:15
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
+++ b/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Книга1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Методологии и проектирование ИС\ДЗ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E2826A-7451-4A3E-9215-2BC00EB1618C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0C228E-D538-4E1A-B035-4F53D465FA74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="2" xr2:uid="{BEBB80D8-0089-49C4-85BD-317F6383F5E1}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="31">
   <si>
     <t>Наименование</t>
   </si>
@@ -55,9 +55,6 @@
     <t>Описание (назначение)</t>
   </si>
   <si>
-    <t>Процессы (работы) диаграммы "Ремонт"</t>
-  </si>
-  <si>
     <t>Диагностирование</t>
   </si>
   <si>
@@ -131,9 +128,6 @@
   </si>
   <si>
     <t>Транспортировка устройства</t>
-  </si>
-  <si>
-    <t>Стрелки диаграммы "Ремонт"</t>
   </si>
   <si>
     <t>Процессы (работы) диаграммы</t>
@@ -915,7 +909,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B1" s="10"/>
     </row>
@@ -929,26 +923,26 @@
     </row>
     <row r="3" spans="1:3" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" s="6"/>
     </row>
     <row r="4" spans="1:3" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="4"/>
     </row>
     <row r="5" spans="1:3" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="8"/>
     </row>
     <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="10"/>
@@ -966,110 +960,110 @@
     </row>
     <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" s="18"/>
       <c r="C10" s="20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" s="18"/>
       <c r="C15" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16" s="18"/>
       <c r="C16" s="19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B18" s="21"/>
       <c r="C18" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" s="24"/>
       <c r="C20" s="25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1092,7 +1086,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B1" s="10"/>
     </row>
@@ -1106,20 +1100,20 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B3" s="6"/>
     </row>
     <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" s="8"/>
     </row>
     <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="10"/>
@@ -1137,83 +1131,83 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="16"/>
       <c r="C8" s="22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="18"/>
       <c r="C9" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="18"/>
       <c r="C10" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="21"/>
       <c r="C15" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B16" s="24"/>
       <c r="C16" s="25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1236,7 +1230,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="B1" s="10"/>
     </row>
@@ -1250,25 +1244,25 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" s="29"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2"/>
     </row>
     <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="8"/>
     </row>
@@ -1293,83 +1287,83 @@
     </row>
     <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="16"/>
       <c r="C10" s="22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15" s="18"/>
       <c r="C15" s="19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="17" t="s">
-        <v>12</v>
+      <c r="A17" s="26" t="s">
+        <v>11</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18" s="24"/>
       <c r="C18" s="25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>